<commit_message>
Limpieza completa: Eliminados archivos MD, test, versiones obsoletas y archivos no conectados
</commit_message>
<xml_diff>
--- a/Full-Agenda/Full.xlsx
+++ b/Full-Agenda/Full.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aramark365-my.sharepoint.com/personal/vega-franco_aramark_cl/Documents/Desktop/Sys_Procesar_Ordenes/Full-Agenda/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dpdhl-my.sharepoint.com/personal/lucas_ezequielg_dhl_com/Documents/Desktop/Sys_Procesar_Ordenes/Full-Agenda/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="92" documentId="13_ncr:1_{CD617C94-7844-4B25-A638-43B0F934D7C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{826C1213-343E-4514-BB5C-1AE40B7F78CE}"/>
+  <xr:revisionPtr revIDLastSave="137" documentId="13_ncr:1_{CD617C94-7844-4B25-A638-43B0F934D7C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{130F2B75-6F3D-4765-8344-EA5A8C3B9A2F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3210" yWindow="-13620" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Full" sheetId="1" r:id="rId1"/>
@@ -19,8 +19,8 @@
     <externalReference r:id="rId2"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Full!$A$1:$Y$1153</definedName>
-    <definedName name="CLSTGO1BFW02_BrandFullWeb_Saturno_CADCOT" localSheetId="0" hidden="1">Full!$A$1:$Y$1153</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Full!$A$1:$Y$1154</definedName>
+    <definedName name="CLSTGO1BFW02_BrandFullWeb_Saturno_CADCOT" localSheetId="0" hidden="1">Full!$A$1:$Y$1154</definedName>
     <definedName name="FULL22" localSheetId="0">Tabla_CLSTGO1BFW02_BrandFullWeb_Saturno_CADCOT10[#All]</definedName>
     <definedName name="FULL22">[1]!Tabla_CLSTGO1BFW02_BrandFullWeb_Saturno_CADCOT[#All]</definedName>
     <definedName name="Fullzona060" localSheetId="0">Tabla_CLSTGO1BFW02_BrandFullWeb_Saturno_CADCOT10[#All]</definedName>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20761" uniqueCount="2884">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20778" uniqueCount="2884">
   <si>
     <t>Fecha Precio</t>
   </si>
@@ -8745,11 +8745,53 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
       <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -8759,11 +8801,17 @@
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
@@ -8922,16 +8970,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla_CLSTGO1BFW02_BrandFullWeb_Saturno_CADCOT10" displayName="Tabla_CLSTGO1BFW02_BrandFullWeb_Saturno_CADCOT10" ref="A1:Y1153" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:Y1153" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla_CLSTGO1BFW02_BrandFullWeb_Saturno_CADCOT10" displayName="Tabla_CLSTGO1BFW02_BrandFullWeb_Saturno_CADCOT10" ref="A1:Y1154" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:Y1154" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}">
     <filterColumn colId="13">
       <filters>
         <filter val="119"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="20">
-      <filters>
-        <filter val="20251231"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -9230,7 +9273,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja13"/>
-  <dimension ref="A1:Y1153"/>
+  <dimension ref="A1:Y1048576"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
@@ -9726,7 +9769,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>20251106</v>
       </c>
@@ -10188,7 +10231,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>20251105</v>
       </c>
@@ -11882,7 +11925,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="35" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>20251105</v>
       </c>
@@ -11959,7 +12002,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="36" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>20251106</v>
       </c>
@@ -12344,7 +12387,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="41" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>20251105</v>
       </c>
@@ -12575,7 +12618,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="44" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>20251106</v>
       </c>
@@ -14269,7 +14312,7 @@
         <v>1639</v>
       </c>
     </row>
-    <row r="66" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>20251106</v>
       </c>
@@ -18042,7 +18085,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="115" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>20251106</v>
       </c>
@@ -18581,7 +18624,7 @@
         <v>2138</v>
       </c>
     </row>
-    <row r="122" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>20251106</v>
       </c>
@@ -23124,7 +23167,7 @@
         <v>2473</v>
       </c>
     </row>
-    <row r="181" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>20251105</v>
       </c>
@@ -23509,7 +23552,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="186" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A186">
         <v>20251105</v>
       </c>
@@ -24202,7 +24245,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="195" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A195">
         <v>20251105</v>
       </c>
@@ -26820,7 +26863,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="229" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A229">
         <v>20251105</v>
       </c>
@@ -30516,7 +30559,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="277" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A277">
         <v>20251105</v>
       </c>
@@ -30747,7 +30790,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="280" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A280">
         <v>20251106</v>
       </c>
@@ -32056,7 +32099,7 @@
         <v>2430</v>
       </c>
     </row>
-    <row r="297" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A297">
         <v>20251203</v>
       </c>
@@ -32133,7 +32176,7 @@
         <v>2430</v>
       </c>
     </row>
-    <row r="298" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A298">
         <v>20251203</v>
       </c>
@@ -35598,7 +35641,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="343" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A343">
         <v>20251105</v>
       </c>
@@ -38601,7 +38644,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="382" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A382">
         <v>20251105</v>
       </c>
@@ -39140,7 +39183,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="389" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A389">
         <v>20251105</v>
       </c>
@@ -39602,7 +39645,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="395" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A395">
         <v>20251106</v>
       </c>
@@ -42682,7 +42725,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="435" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="435" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A435">
         <v>20251105</v>
       </c>
@@ -47071,7 +47114,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="492" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="492" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A492">
         <v>20251106</v>
       </c>
@@ -49304,7 +49347,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="521" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="521" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A521">
         <v>20251105</v>
       </c>
@@ -49535,7 +49578,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="524" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="524" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A524">
         <v>20251105</v>
       </c>
@@ -51922,7 +51965,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="555" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="555" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A555">
         <v>20251105</v>
       </c>
@@ -52307,7 +52350,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="560" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="560" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A560">
         <v>20251106</v>
       </c>
@@ -53154,7 +53197,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="571" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="571" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A571">
         <v>20251106</v>
       </c>
@@ -53385,7 +53428,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="574" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="574" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A574">
         <v>20251105</v>
       </c>
@@ -53616,7 +53659,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="577" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="577" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A577">
         <v>20251105</v>
       </c>
@@ -53924,7 +53967,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="581" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="581" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A581">
         <v>20251105</v>
       </c>
@@ -54155,7 +54198,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="584" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="584" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A584">
         <v>20251118</v>
       </c>
@@ -55387,7 +55430,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="600" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="600" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A600">
         <v>20251105</v>
       </c>
@@ -55464,7 +55507,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="601" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="601" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A601">
         <v>20251106</v>
       </c>
@@ -59391,7 +59434,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="652" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="652" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A652">
         <v>20251118</v>
       </c>
@@ -62702,7 +62745,7 @@
         <v>782</v>
       </c>
     </row>
-    <row r="695" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="695" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A695">
         <v>20251118</v>
       </c>
@@ -63241,7 +63284,7 @@
         <v>782</v>
       </c>
     </row>
-    <row r="702" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="702" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A702">
         <v>20251106</v>
       </c>
@@ -64088,7 +64131,7 @@
         <v>782</v>
       </c>
     </row>
-    <row r="713" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="713" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A713">
         <v>20251106</v>
       </c>
@@ -67245,7 +67288,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="754" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="754" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A754">
         <v>20251106</v>
       </c>
@@ -68323,7 +68366,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="768" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="768" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A768">
         <v>20251105</v>
       </c>
@@ -68477,7 +68520,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="770" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="770" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A770">
         <v>20251105</v>
       </c>
@@ -68785,7 +68828,7 @@
         <v>862</v>
       </c>
     </row>
-    <row r="774" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="774" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A774">
         <v>20251106</v>
       </c>
@@ -69401,7 +69444,7 @@
         <v>862</v>
       </c>
     </row>
-    <row r="782" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="782" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A782">
         <v>20251106</v>
       </c>
@@ -71634,7 +71677,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="811" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="811" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A811">
         <v>20251106</v>
       </c>
@@ -72096,7 +72139,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="817" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="817" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A817">
         <v>20251105</v>
       </c>
@@ -72250,7 +72293,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="819" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="819" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A819">
         <v>20251105</v>
       </c>
@@ -73559,7 +73602,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="836" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="836" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A836">
         <v>20251105</v>
       </c>
@@ -73790,7 +73833,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="839" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="839" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A839">
         <v>20251105</v>
       </c>
@@ -78025,7 +78068,7 @@
         <v>946</v>
       </c>
     </row>
-    <row r="894" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="894" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A894">
         <v>20251106</v>
       </c>
@@ -79719,7 +79762,7 @@
         <v>964</v>
       </c>
     </row>
-    <row r="916" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="916" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A916">
         <v>20251202</v>
       </c>
@@ -82722,7 +82765,7 @@
         <v>946</v>
       </c>
     </row>
-    <row r="955" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="955" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A955">
         <v>20251105</v>
       </c>
@@ -82953,7 +82996,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="958" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="958" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A958">
         <v>20251106</v>
       </c>
@@ -83261,7 +83304,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="962" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="962" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A962">
         <v>20251106</v>
       </c>
@@ -83492,7 +83535,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="965" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="965" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A965">
         <v>20251106</v>
       </c>
@@ -83646,7 +83689,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="967" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="967" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A967">
         <v>20251105</v>
       </c>
@@ -83954,7 +83997,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="971" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="971" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A971">
         <v>20251106</v>
       </c>
@@ -84185,7 +84228,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="974" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="974" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A974">
         <v>20251106</v>
       </c>
@@ -84416,7 +84459,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="977" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="977" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A977">
         <v>20251106</v>
       </c>
@@ -84647,7 +84690,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="980" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="980" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A980">
         <v>20251106</v>
       </c>
@@ -84955,7 +84998,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="984" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="984" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A984">
         <v>20251106</v>
       </c>
@@ -85109,7 +85152,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="986" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="986" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A986">
         <v>20251106</v>
       </c>
@@ -85494,7 +85537,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="991" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="991" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A991">
         <v>20251106</v>
       </c>
@@ -85802,7 +85845,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="995" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="995" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A995">
         <v>20251106</v>
       </c>
@@ -86187,7 +86230,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="1000" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1000" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1000">
         <v>20251105</v>
       </c>
@@ -86341,7 +86384,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="1002" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1002" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1002">
         <v>20251105</v>
       </c>
@@ -86572,7 +86615,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="1005" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1005" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1005">
         <v>20251106</v>
       </c>
@@ -86880,7 +86923,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="1009" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1009" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1009">
         <v>20251106</v>
       </c>
@@ -87111,7 +87154,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="1012" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1012" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1012">
         <v>20251105</v>
       </c>
@@ -88497,7 +88540,7 @@
         <v>1084</v>
       </c>
     </row>
-    <row r="1030" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1030" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1030">
         <v>20251106</v>
       </c>
@@ -92655,7 +92698,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="1084" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1084" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1084">
         <v>20251105</v>
       </c>
@@ -93579,7 +93622,7 @@
         <v>1203</v>
       </c>
     </row>
-    <row r="1096" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1096" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1096">
         <v>20251106</v>
       </c>
@@ -93887,7 +93930,7 @@
         <v>840</v>
       </c>
     </row>
-    <row r="1100" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1100" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1100">
         <v>20251106</v>
       </c>
@@ -94041,7 +94084,7 @@
         <v>840</v>
       </c>
     </row>
-    <row r="1102" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1102" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1102">
         <v>20251106</v>
       </c>
@@ -94195,7 +94238,7 @@
         <v>840</v>
       </c>
     </row>
-    <row r="1104" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1104" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1104">
         <v>20251106</v>
       </c>
@@ -94349,7 +94392,7 @@
         <v>840</v>
       </c>
     </row>
-    <row r="1106" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1106" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1106">
         <v>20251106</v>
       </c>
@@ -94811,7 +94854,7 @@
         <v>840</v>
       </c>
     </row>
-    <row r="1112" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1112" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1112">
         <v>20251106</v>
       </c>
@@ -95581,7 +95624,7 @@
         <v>840</v>
       </c>
     </row>
-    <row r="1122" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1122" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1122">
         <v>20251106</v>
       </c>
@@ -97737,7 +97780,7 @@
         <v>840</v>
       </c>
     </row>
-    <row r="1150" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1150" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1150">
         <v>20251105</v>
       </c>
@@ -98044,6 +98087,86 @@
       <c r="Y1153" t="s">
         <v>840</v>
       </c>
+    </row>
+    <row r="1154" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A1154" s="5">
+        <v>20251120</v>
+      </c>
+      <c r="B1154" s="6" t="s">
+        <v>1768</v>
+      </c>
+      <c r="C1154">
+        <v>100042</v>
+      </c>
+      <c r="D1154" s="6" t="s">
+        <v>1769</v>
+      </c>
+      <c r="E1154" s="6" t="s">
+        <v>2423</v>
+      </c>
+      <c r="F1154" s="6" t="s">
+        <v>2730</v>
+      </c>
+      <c r="G1154" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1154" s="6" t="s">
+        <v>1300</v>
+      </c>
+      <c r="I1154" s="6" t="s">
+        <v>1301</v>
+      </c>
+      <c r="J1154" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K1154" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="L1154" s="6" t="s">
+        <v>391</v>
+      </c>
+      <c r="M1154" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="N1154" s="6" t="s">
+        <v>1392</v>
+      </c>
+      <c r="O1154" s="6" t="s">
+        <v>1393</v>
+      </c>
+      <c r="P1154" s="7">
+        <v>9500</v>
+      </c>
+      <c r="Q1154" s="8">
+        <v>15696</v>
+      </c>
+      <c r="R1154" s="8">
+        <v>436</v>
+      </c>
+      <c r="S1154" s="6">
+        <v>0</v>
+      </c>
+      <c r="T1154" s="6">
+        <v>20251201</v>
+      </c>
+      <c r="U1154" s="6">
+        <v>20251231</v>
+      </c>
+      <c r="V1154" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="W1154" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="X1154" s="6" t="s">
+        <v>839</v>
+      </c>
+      <c r="Y1154" s="9" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="1048576" spans="21:21" x14ac:dyDescent="0.25">
+      <c r="U1048576" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -98056,6 +98179,11 @@
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="5acfaaec-c0b5-444f-b194-f67401ef1536" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
@@ -98063,12 +98191,18 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="5acfaaec-c0b5-444f-b194-f67401ef1536" ContentTypeId="0x0101" PreviousValue="false"/>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="52c65fac-2f2f-421c-b176-d18632a0be36" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4b69a02c-d85f-4df0-8349-74540ec962fe">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100505D21C870C1944596134F8CDF91CFA3" ma:contentTypeVersion="14" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="0a35f0eacab48321e7390866c63086ee">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4b69a02c-d85f-4df0-8349-74540ec962fe" xmlns:ns3="52c65fac-2f2f-421c-b176-d18632a0be36" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="95e20a23532cedf7941895a3f3e2ccf1" ns2:_="" ns3:_="">
     <xsd:import namespace="4b69a02c-d85f-4df0-8349-74540ec962fe"/>
@@ -98257,18 +98391,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="52c65fac-2f2f-421c-b176-d18632a0be36" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4b69a02c-d85f-4df0-8349-74540ec962fe">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3964F27B-C9A8-43EE-B2E5-9A3158CC5E65}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BF1CE709-AE3D-464E-804F-6C5D70B843F2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -98276,15 +98407,18 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3964F27B-C9A8-43EE-B2E5-9A3158CC5E65}">
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4D2EB95-62A5-4AAC-9A91-068B01E668F1}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="52c65fac-2f2f-421c-b176-d18632a0be36"/>
+    <ds:schemaRef ds:uri="4b69a02c-d85f-4df0-8349-74540ec962fe"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6244816-A925-4667-8E5A-F2CCD75B6327}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -98303,20 +98437,9 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4D2EB95-62A5-4AAC-9A91-068B01E668F1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="52c65fac-2f2f-421c-b176-d18632a0be36"/>
-    <ds:schemaRef ds:uri="4b69a02c-d85f-4df0-8349-74540ec962fe"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{736915f3-2f02-4945-8997-f2963298db46}" enabled="1" method="Standard" siteId="{cd99fef8-1cd3-4a2a-9bdf-15531181d65e}" removed="0"/>
   <clbl:label id="{b1519f0f-2dbf-4e21-bf34-a686ce97588a}" enabled="0" method="" siteId="{b1519f0f-2dbf-4e21-bf34-a686ce97588a}" removed="1"/>
-  <clbl:label id="{cd99fef8-1cd3-4a2a-9bdf-15531181d65e}" enabled="0" method="" siteId="{cd99fef8-1cd3-4a2a-9bdf-15531181d65e}" removed="1"/>
 </clbl:labelList>
 </file>
</xml_diff>